<commit_message>
#3 Updated Client BOM!
</commit_message>
<xml_diff>
--- a/Design-Files/FMM-v1.0/BOM/Client-BOM-FMM-v1.0.xlsx
+++ b/Design-Files/FMM-v1.0/BOM/Client-BOM-FMM-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="435">
   <si>
     <t>#</t>
   </si>
@@ -1315,6 +1315,15 @@
   </si>
   <si>
     <t>R2, R69</t>
+  </si>
+  <si>
+    <t>Voltlink</t>
+  </si>
+  <si>
+    <t>Tinde</t>
+  </si>
+  <si>
+    <t>VoltLink CP2102N USB Serial Adapter &amp; Programmer</t>
   </si>
 </sst>
 </file>
@@ -1699,7 +1708,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1760,13 +1769,7 @@
     <xf numFmtId="164" fontId="8" fillId="3" borderId="13" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1811,13 +1814,25 @@
     <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1846,21 +1861,6 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2150,7 +2150,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:W100"/>
+  <dimension ref="A1:Z101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -2168,10 +2168,13 @@
     <col min="14" max="14" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="29.42578125" customWidth="1"/>
     <col min="16" max="16" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="36" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2180,15 +2183,17 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-    </row>
-    <row r="2" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+    </row>
+    <row r="2" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -2220,7 +2225,7 @@
       <c r="K2" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="L2" s="28" t="s">
+      <c r="L2" s="26" t="s">
         <v>335</v>
       </c>
       <c r="M2" s="5" t="s">
@@ -2233,7 +2238,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -2267,19 +2272,31 @@
         <f>J3*5</f>
         <v>45</v>
       </c>
-      <c r="L3" s="29" t="s">
+      <c r="L3" s="27" t="s">
         <v>337</v>
       </c>
       <c r="M3" s="14">
         <v>0.124</v>
       </c>
-      <c r="N3" s="37">
+      <c r="N3" s="35">
         <f>M3*K3</f>
         <v>5.58</v>
       </c>
       <c r="O3" s="7"/>
-    </row>
-    <row r="4" spans="1:15" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T3" t="b">
+        <f>IF(Q3=D3,TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="U3" t="b">
+        <f>IF(R3=G3,TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="V3" t="b">
+        <f>IF(S3=J3,TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B93" si="0">ROW(B4) - ROW($B$2)</f>
@@ -2313,19 +2330,31 @@
         <f t="shared" ref="K4:K68" si="1">J4*5</f>
         <v>155</v>
       </c>
-      <c r="L4" s="30" t="s">
+      <c r="L4" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M4" s="14">
         <v>1.9400000000000001E-2</v>
       </c>
-      <c r="N4" s="37">
+      <c r="N4" s="35">
         <f t="shared" ref="N4:N74" si="2">M4*K4</f>
         <v>3.0070000000000001</v>
       </c>
       <c r="O4" s="9"/>
-    </row>
-    <row r="5" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T4" t="b">
+        <f t="shared" ref="T4:T67" si="3">IF(Q4=D4,TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="U4" t="b">
+        <f t="shared" ref="U4:U67" si="4">IF(R4=G4,TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="V4" t="b">
+        <f t="shared" ref="V4:V67" si="5">IF(S4=J4,TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -2359,19 +2388,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L5" s="30" t="s">
+      <c r="L5" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M5" s="14">
         <v>0.92100000000000004</v>
       </c>
-      <c r="N5" s="37">
+      <c r="N5" s="35">
         <f t="shared" si="2"/>
         <v>9.2100000000000009</v>
       </c>
       <c r="O5" s="7"/>
-    </row>
-    <row r="6" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T5" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U5" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V5" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -2405,19 +2446,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L6" s="30" t="s">
+      <c r="L6" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M6" s="14">
         <v>1.0389999999999999</v>
       </c>
-      <c r="N6" s="37">
+      <c r="N6" s="35">
         <f t="shared" si="2"/>
         <v>10.389999999999999</v>
       </c>
       <c r="O6" s="9"/>
-    </row>
-    <row r="7" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T6" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U6" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V6" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -2451,19 +2504,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L7" s="30" t="s">
+      <c r="L7" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M7" s="14">
         <v>0.22</v>
       </c>
-      <c r="N7" s="37">
+      <c r="N7" s="35">
         <f t="shared" si="2"/>
         <v>2.2000000000000002</v>
       </c>
       <c r="O7" s="7"/>
-    </row>
-    <row r="8" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T7" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U7" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V7" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -2497,19 +2562,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L8" s="30" t="s">
+      <c r="L8" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M8" s="14">
         <v>0.1</v>
       </c>
-      <c r="N8" s="37">
+      <c r="N8" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O8" s="9"/>
-    </row>
-    <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T8" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U8" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V8" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -2543,19 +2620,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L9" s="30" t="s">
+      <c r="L9" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M9" s="14">
         <v>0.1</v>
       </c>
-      <c r="N9" s="37">
+      <c r="N9" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O9" s="7"/>
-    </row>
-    <row r="10" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T9" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U9" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V9" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -2589,19 +2678,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L10" s="30" t="s">
+      <c r="L10" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M10" s="14">
         <v>0.1</v>
       </c>
-      <c r="N10" s="37">
+      <c r="N10" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O10" s="9"/>
-    </row>
-    <row r="11" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T10" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U10" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V10" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -2635,19 +2736,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L11" s="30" t="s">
+      <c r="L11" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M11" s="14">
         <v>0.1</v>
       </c>
-      <c r="N11" s="37">
+      <c r="N11" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O11" s="7"/>
-    </row>
-    <row r="12" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T11" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U11" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V11" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -2681,19 +2794,31 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="L12" s="30" t="s">
+      <c r="L12" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M12" s="14">
         <v>0.22600000000000001</v>
       </c>
-      <c r="N12" s="37">
+      <c r="N12" s="35">
         <f t="shared" si="2"/>
         <v>3.39</v>
       </c>
       <c r="O12" s="9"/>
-    </row>
-    <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T12" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U12" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V12" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -2727,19 +2852,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L13" s="30" t="s">
+      <c r="L13" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M13" s="14">
         <v>0.73699999999999999</v>
       </c>
-      <c r="N13" s="37">
+      <c r="N13" s="35">
         <f t="shared" si="2"/>
         <v>7.37</v>
       </c>
       <c r="O13" s="7"/>
-    </row>
-    <row r="14" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T13" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U13" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V13" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -2773,19 +2910,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L14" s="30" t="s">
+      <c r="L14" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M14" s="14">
         <v>0.22</v>
       </c>
-      <c r="N14" s="37">
+      <c r="N14" s="35">
         <f t="shared" si="2"/>
         <v>1.1000000000000001</v>
       </c>
       <c r="O14" s="9"/>
-    </row>
-    <row r="15" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T14" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U14" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V14" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -2819,19 +2968,31 @@
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
-      <c r="L15" s="30" t="s">
+      <c r="L15" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M15" s="14">
         <v>0.26</v>
       </c>
-      <c r="N15" s="37">
+      <c r="N15" s="35">
         <f t="shared" si="2"/>
         <v>9.1</v>
       </c>
       <c r="O15" s="7"/>
-    </row>
-    <row r="16" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T15" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U15" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V15" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -2865,19 +3026,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L16" s="30" t="s">
+      <c r="L16" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M16" s="14">
         <v>0.45</v>
       </c>
-      <c r="N16" s="37">
+      <c r="N16" s="35">
         <f t="shared" si="2"/>
         <v>2.25</v>
       </c>
       <c r="O16" s="9"/>
-    </row>
-    <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T16" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U16" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V16" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -2911,19 +3084,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L17" s="30" t="s">
+      <c r="L17" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M17" s="14">
         <v>0.11899999999999999</v>
       </c>
-      <c r="N17" s="37">
+      <c r="N17" s="35">
         <f t="shared" si="2"/>
         <v>1.19</v>
       </c>
       <c r="O17" s="7"/>
-    </row>
-    <row r="18" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T17" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U17" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V17" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -2957,19 +3142,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L18" s="30" t="s">
+      <c r="L18" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M18" s="14">
         <v>0.48</v>
       </c>
-      <c r="N18" s="37">
+      <c r="N18" s="35">
         <f t="shared" si="2"/>
         <v>2.4</v>
       </c>
       <c r="O18" s="9"/>
-    </row>
-    <row r="19" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T18" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U18" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V18" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -3003,22 +3200,34 @@
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
-      <c r="L19" s="30" t="s">
+      <c r="L19" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M19" s="14">
         <v>0.1</v>
       </c>
-      <c r="N19" s="37">
+      <c r="N19" s="35">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="O19" s="7"/>
-    </row>
-    <row r="20" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T19" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U19" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V19" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
-        <f t="shared" ref="B20" si="3">ROW(B20) - ROW($B$2)</f>
+        <f t="shared" ref="B20" si="6">ROW(B20) - ROW($B$2)</f>
         <v>18</v>
       </c>
       <c r="C20" s="13" t="s">
@@ -3049,19 +3258,31 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L20" s="30" t="s">
+      <c r="L20" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M20" s="14">
         <v>0.1</v>
       </c>
-      <c r="N20" s="37">
+      <c r="N20" s="35">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="O20" s="7"/>
-    </row>
-    <row r="21" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T20" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U20" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V20" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -3095,22 +3316,34 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L21" s="30" t="s">
+      <c r="L21" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M21" s="14">
         <v>0.1</v>
       </c>
-      <c r="N21" s="37">
+      <c r="N21" s="35">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="O21" s="7"/>
-    </row>
-    <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T21" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U21" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V21" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
-        <f t="shared" ref="B22" si="4">ROW(B22) - ROW($B$2)</f>
+        <f t="shared" ref="B22" si="7">ROW(B22) - ROW($B$2)</f>
         <v>20</v>
       </c>
       <c r="C22" s="13" t="s">
@@ -3141,19 +3374,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L22" s="30" t="s">
+      <c r="L22" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M22" s="14">
         <v>0.37</v>
       </c>
-      <c r="N22" s="37">
+      <c r="N22" s="35">
         <f t="shared" si="2"/>
         <v>1.85</v>
       </c>
       <c r="O22" s="7"/>
-    </row>
-    <row r="23" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T22" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U22" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V22" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -3187,19 +3432,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L23" s="30" t="s">
+      <c r="L23" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M23" s="14">
         <v>2.96</v>
       </c>
-      <c r="N23" s="37">
+      <c r="N23" s="35">
         <f t="shared" si="2"/>
         <v>14.8</v>
       </c>
       <c r="O23" s="7"/>
-    </row>
-    <row r="24" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T23" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U23" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V23" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -3233,19 +3490,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L24" s="30" t="s">
+      <c r="L24" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M24" s="14">
         <v>0.91</v>
       </c>
-      <c r="N24" s="37">
+      <c r="N24" s="35">
         <f t="shared" si="2"/>
         <v>4.55</v>
       </c>
       <c r="O24" s="9"/>
-    </row>
-    <row r="25" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T24" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U24" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V24" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -3279,19 +3548,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L25" s="30" t="s">
+      <c r="L25" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M25" s="14">
         <v>0.21</v>
       </c>
-      <c r="N25" s="37">
+      <c r="N25" s="35">
         <f t="shared" si="2"/>
         <v>1.05</v>
       </c>
       <c r="O25" s="7"/>
-    </row>
-    <row r="26" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T25" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U25" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V25" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -3325,19 +3606,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L26" s="30" t="s">
+      <c r="L26" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M26" s="14">
         <v>0.38</v>
       </c>
-      <c r="N26" s="37">
+      <c r="N26" s="35">
         <f t="shared" si="2"/>
         <v>1.9</v>
       </c>
       <c r="O26" s="9"/>
-    </row>
-    <row r="27" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T26" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U26" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V26" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -3371,19 +3664,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L27" s="30" t="s">
+      <c r="L27" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M27" s="14">
         <v>0.255</v>
       </c>
-      <c r="N27" s="37">
+      <c r="N27" s="35">
         <f t="shared" si="2"/>
         <v>2.5499999999999998</v>
       </c>
       <c r="O27" s="7"/>
-    </row>
-    <row r="28" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T27" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U27" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V27" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -3392,45 +3697,57 @@
       <c r="C28" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D28" s="50" t="s">
+      <c r="D28" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="E28" s="50" t="s">
+      <c r="E28" s="40" t="s">
         <v>113</v>
       </c>
-      <c r="F28" s="50" t="s">
+      <c r="F28" s="40" t="s">
         <v>178</v>
       </c>
-      <c r="G28" s="51" t="s">
+      <c r="G28" s="41" t="s">
         <v>225</v>
       </c>
-      <c r="H28" s="50" t="s">
+      <c r="H28" s="40" t="s">
         <v>277</v>
       </c>
-      <c r="I28" s="52" t="s">
+      <c r="I28" s="42" t="s">
         <v>336</v>
       </c>
-      <c r="J28" s="50">
+      <c r="J28" s="40">
         <v>1</v>
       </c>
-      <c r="K28" s="53">
+      <c r="K28" s="43">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L28" s="30" t="s">
+      <c r="L28" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M28" s="14" t="s">
         <v>336</v>
       </c>
-      <c r="N28" s="37" t="s">
+      <c r="N28" s="35" t="s">
         <v>336</v>
       </c>
-      <c r="O28" s="49" t="s">
+      <c r="O28" s="39" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T28" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U28" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V28" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -3464,19 +3781,31 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="L29" s="30" t="s">
+      <c r="L29" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M29" s="14">
         <v>1.54E-2</v>
       </c>
-      <c r="N29" s="37">
+      <c r="N29" s="35">
         <f t="shared" si="2"/>
         <v>0.23100000000000001</v>
       </c>
       <c r="O29" s="7"/>
-    </row>
-    <row r="30" spans="1:15" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T29" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U29" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V29" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
@@ -3510,19 +3839,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L30" s="30" t="s">
+      <c r="L30" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M30" s="14">
         <v>1.5</v>
       </c>
-      <c r="N30" s="37">
+      <c r="N30" s="35">
         <f t="shared" si="2"/>
         <v>7.5</v>
       </c>
       <c r="O30" s="9"/>
-    </row>
-    <row r="31" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T30" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U30" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V30" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
@@ -3556,19 +3897,31 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L31" s="30" t="s">
+      <c r="L31" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M31" s="14">
         <v>0.26900000000000002</v>
       </c>
-      <c r="N31" s="37">
+      <c r="N31" s="35">
         <f t="shared" si="2"/>
         <v>5.3800000000000008</v>
       </c>
       <c r="O31" s="7"/>
-    </row>
-    <row r="32" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T31" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U31" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V31" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f>ROW(B32) - ROW($B$2)</f>
@@ -3602,19 +3955,31 @@
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="L32" s="30" t="s">
+      <c r="L32" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M32" s="14">
         <v>9.2999999999999999E-2</v>
       </c>
-      <c r="N32" s="37">
+      <c r="N32" s="35">
         <f t="shared" si="2"/>
         <v>2.3250000000000002</v>
       </c>
       <c r="O32" s="7"/>
-    </row>
-    <row r="33" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T32" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U32" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V32" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f t="shared" si="0"/>
@@ -3648,19 +4013,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L33" s="30" t="s">
+      <c r="L33" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M33" s="14">
         <v>4.3280000000000003</v>
       </c>
-      <c r="N33" s="37">
+      <c r="N33" s="35">
         <f t="shared" si="2"/>
         <v>21.64</v>
       </c>
       <c r="O33" s="9"/>
-    </row>
-    <row r="34" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T33" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U33" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V33" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f>ROW(B34) - ROW($B$2)</f>
@@ -3694,19 +4071,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L34" s="30" t="s">
+      <c r="L34" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M34" s="14">
         <v>0.3725</v>
       </c>
-      <c r="N34" s="37">
+      <c r="N34" s="35">
         <f t="shared" si="2"/>
         <v>1.8625</v>
       </c>
       <c r="O34" s="7"/>
-    </row>
-    <row r="35" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T34" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U34" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V34" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f t="shared" si="0"/>
@@ -3740,19 +4129,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L35" s="30" t="s">
+      <c r="L35" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M35" s="14">
         <v>0.57599999999999996</v>
       </c>
-      <c r="N35" s="37">
+      <c r="N35" s="35">
         <f t="shared" si="2"/>
         <v>2.88</v>
       </c>
       <c r="O35" s="9"/>
-    </row>
-    <row r="36" spans="1:15" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T35" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U35" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V35" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
         <f>ROW(B36) - ROW($B$2)</f>
@@ -3786,19 +4187,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L36" s="30" t="s">
+      <c r="L36" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M36" s="14">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="N36" s="37">
+      <c r="N36" s="35">
         <f t="shared" si="2"/>
         <v>0.34</v>
       </c>
       <c r="O36" s="7"/>
-    </row>
-    <row r="37" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T36" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U36" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V36" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
         <f t="shared" si="0"/>
@@ -3832,19 +4245,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L37" s="30" t="s">
+      <c r="L37" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M37" s="14">
         <v>25.25</v>
       </c>
-      <c r="N37" s="37">
+      <c r="N37" s="35">
         <f t="shared" si="2"/>
         <v>126.25</v>
       </c>
       <c r="O37" s="9"/>
-    </row>
-    <row r="38" spans="1:15" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T37" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U37" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V37" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
         <f>ROW(B38) - ROW($B$2)</f>
@@ -3878,19 +4303,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L38" s="30" t="s">
+      <c r="L38" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M38" s="14">
         <v>0.30809999999999998</v>
       </c>
-      <c r="N38" s="37">
+      <c r="N38" s="35">
         <f t="shared" si="2"/>
         <v>3.081</v>
       </c>
       <c r="O38" s="7"/>
-    </row>
-    <row r="39" spans="1:15" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T38" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U38" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V38" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
         <f t="shared" si="0"/>
@@ -3924,19 +4361,31 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L39" s="30" t="s">
+      <c r="L39" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M39" s="14">
         <v>0.30669999999999997</v>
       </c>
-      <c r="N39" s="37">
+      <c r="N39" s="35">
         <f t="shared" si="2"/>
         <v>6.1339999999999995</v>
       </c>
       <c r="O39" s="9"/>
-    </row>
-    <row r="40" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T39" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U39" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V39" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
         <f>ROW(B40) - ROW($B$2)</f>
@@ -3970,19 +4419,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L40" s="30" t="s">
+      <c r="L40" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M40" s="14">
         <v>1.56</v>
       </c>
-      <c r="N40" s="37">
+      <c r="N40" s="35">
         <f t="shared" si="2"/>
         <v>7.8000000000000007</v>
       </c>
       <c r="O40" s="7"/>
-    </row>
-    <row r="41" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T40" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U40" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V40" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
         <f t="shared" si="0"/>
@@ -4016,19 +4477,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L41" s="30" t="s">
+      <c r="L41" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M41" s="14">
         <v>1.19</v>
       </c>
-      <c r="N41" s="37">
+      <c r="N41" s="35">
         <f t="shared" si="2"/>
         <v>5.9499999999999993</v>
       </c>
       <c r="O41" s="9"/>
-    </row>
-    <row r="42" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T41" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U41" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V41" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="11">
         <f>ROW(B42) - ROW($B$2)</f>
@@ -4062,19 +4535,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L42" s="30" t="s">
+      <c r="L42" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M42" s="14">
         <v>1.85</v>
       </c>
-      <c r="N42" s="37">
+      <c r="N42" s="35">
         <f t="shared" si="2"/>
         <v>9.25</v>
       </c>
       <c r="O42" s="7"/>
-    </row>
-    <row r="43" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T42" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U42" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V42" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
         <f t="shared" si="0"/>
@@ -4108,19 +4593,31 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L43" s="30" t="s">
+      <c r="L43" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M43" s="14">
         <v>2.0799999999999999E-2</v>
       </c>
-      <c r="N43" s="37">
+      <c r="N43" s="35">
         <f t="shared" si="2"/>
         <v>0.41599999999999998</v>
       </c>
       <c r="O43" s="9"/>
-    </row>
-    <row r="44" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T43" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U43" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V43" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
         <f>ROW(B44) - ROW($B$2)</f>
@@ -4154,19 +4651,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L44" s="30" t="s">
+      <c r="L44" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M44" s="14">
         <v>2.1700000000000001E-2</v>
       </c>
-      <c r="N44" s="37">
+      <c r="N44" s="35">
         <f t="shared" si="2"/>
         <v>0.217</v>
       </c>
       <c r="O44" s="7"/>
-    </row>
-    <row r="45" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T44" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U44" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V44" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
         <f t="shared" si="0"/>
@@ -4200,19 +4709,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L45" s="30" t="s">
+      <c r="L45" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M45" s="14">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="N45" s="37">
+      <c r="N45" s="35">
         <f t="shared" si="2"/>
         <v>0.10999999999999999</v>
       </c>
       <c r="O45" s="9"/>
-    </row>
-    <row r="46" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T45" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U45" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V45" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
         <f>ROW(B46) - ROW($B$2)</f>
@@ -4246,19 +4767,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L46" s="30" t="s">
+      <c r="L46" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M46" s="14">
         <v>3.1300000000000001E-2</v>
       </c>
-      <c r="N46" s="37">
+      <c r="N46" s="35">
         <f t="shared" si="2"/>
         <v>0.1565</v>
       </c>
       <c r="O46" s="7"/>
-    </row>
-    <row r="47" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T46" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U46" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V46" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
         <f t="shared" si="0"/>
@@ -4292,19 +4825,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L47" s="30" t="s">
+      <c r="L47" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M47" s="14">
         <v>1.0900000000000001</v>
       </c>
-      <c r="N47" s="37">
+      <c r="N47" s="35">
         <f t="shared" si="2"/>
         <v>5.45</v>
       </c>
       <c r="O47" s="9"/>
-    </row>
-    <row r="48" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T47" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U47" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V47" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
         <f>ROW(B48) - ROW($B$2)</f>
@@ -4338,19 +4883,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L48" s="30" t="s">
+      <c r="L48" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M48" s="14">
         <v>1.0900000000000001</v>
       </c>
-      <c r="N48" s="37">
+      <c r="N48" s="35">
         <f t="shared" si="2"/>
         <v>5.45</v>
       </c>
       <c r="O48" s="7"/>
-    </row>
-    <row r="49" spans="1:15" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T48" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U48" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V48" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
         <f t="shared" si="0"/>
@@ -4384,19 +4941,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L49" s="30" t="s">
+      <c r="L49" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M49" s="14">
         <v>0.2</v>
       </c>
-      <c r="N49" s="37">
+      <c r="N49" s="35">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="O49" s="9"/>
-    </row>
-    <row r="50" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T49" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U49" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V49" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
         <f t="shared" si="0"/>
@@ -4430,19 +4999,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L50" s="30" t="s">
+      <c r="L50" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M50" s="14">
         <v>0.15</v>
       </c>
-      <c r="N50" s="37">
+      <c r="N50" s="35">
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
       <c r="O50" s="9"/>
-    </row>
-    <row r="51" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T50" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U50" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V50" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="11">
         <f>ROW(B51) - ROW($B$2)</f>
@@ -4476,19 +5057,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L51" s="30" t="s">
+      <c r="L51" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M51" s="14">
         <v>0.1</v>
       </c>
-      <c r="N51" s="37">
+      <c r="N51" s="35">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="O51" s="7"/>
-    </row>
-    <row r="52" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T51" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U51" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V51" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="11">
         <f t="shared" si="0"/>
@@ -4522,19 +5115,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L52" s="30" t="s">
+      <c r="L52" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M52" s="14">
         <v>0.15</v>
       </c>
-      <c r="N52" s="37">
+      <c r="N52" s="35">
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
       <c r="O52" s="9"/>
-    </row>
-    <row r="53" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T52" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U52" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V52" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="11">
         <f>ROW(B53) - ROW($B$2)</f>
@@ -4568,19 +5173,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L53" s="30" t="s">
+      <c r="L53" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M53" s="14">
         <v>0.13</v>
       </c>
-      <c r="N53" s="37">
+      <c r="N53" s="35">
         <f t="shared" si="2"/>
         <v>0.65</v>
       </c>
       <c r="O53" s="7"/>
-    </row>
-    <row r="54" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T53" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U53" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V53" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="11">
         <f t="shared" si="0"/>
@@ -4614,19 +5231,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L54" s="30" t="s">
+      <c r="L54" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M54" s="14">
         <v>0.64</v>
       </c>
-      <c r="N54" s="37">
+      <c r="N54" s="35">
         <f t="shared" si="2"/>
         <v>3.2</v>
       </c>
       <c r="O54" s="9"/>
-    </row>
-    <row r="55" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T54" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U54" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V54" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
         <f>ROW(B55) - ROW($B$2)</f>
@@ -4660,19 +5289,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L55" s="30" t="s">
+      <c r="L55" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M55" s="14">
         <v>0.15</v>
       </c>
-      <c r="N55" s="37">
+      <c r="N55" s="35">
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
       <c r="O55" s="7"/>
-    </row>
-    <row r="56" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T55" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U55" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V55" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
         <f t="shared" si="0"/>
@@ -4706,19 +5347,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L56" s="30" t="s">
+      <c r="L56" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M56" s="14">
         <v>0.15</v>
       </c>
-      <c r="N56" s="37">
+      <c r="N56" s="35">
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
       <c r="O56" s="9"/>
-    </row>
-    <row r="57" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T56" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U56" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V56" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
         <f>ROW(B57) - ROW($B$2)</f>
@@ -4752,19 +5405,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L57" s="30" t="s">
+      <c r="L57" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M57" s="14">
         <v>0.15</v>
       </c>
-      <c r="N57" s="37">
+      <c r="N57" s="35">
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
       <c r="O57" s="7"/>
-    </row>
-    <row r="58" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T57" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U57" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V57" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
         <f t="shared" si="0"/>
@@ -4798,19 +5463,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L58" s="30" t="s">
+      <c r="L58" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M58" s="14">
         <v>0.15</v>
       </c>
-      <c r="N58" s="37">
+      <c r="N58" s="35">
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
       <c r="O58" s="9"/>
-    </row>
-    <row r="59" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T58" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U58" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V58" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="11">
         <f>ROW(B59) - ROW($B$2)</f>
@@ -4844,19 +5521,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L59" s="30" t="s">
+      <c r="L59" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M59" s="14">
         <v>0.1</v>
       </c>
-      <c r="N59" s="37">
+      <c r="N59" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O59" s="7"/>
-    </row>
-    <row r="60" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T59" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U59" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V59" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="11">
         <f t="shared" si="0"/>
@@ -4890,19 +5579,31 @@
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="L60" s="30" t="s">
+      <c r="L60" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M60" s="14">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="N60" s="37">
+      <c r="N60" s="35">
         <f t="shared" si="2"/>
         <v>0.375</v>
       </c>
       <c r="O60" s="9"/>
-    </row>
-    <row r="61" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T60" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U60" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V60" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="11">
         <f>ROW(B61) - ROW($B$2)</f>
@@ -4936,19 +5637,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L61" s="30" t="s">
+      <c r="L61" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M61" s="14">
         <v>0.1</v>
       </c>
-      <c r="N61" s="37">
+      <c r="N61" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O61" s="7"/>
-    </row>
-    <row r="62" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T61" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U61" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V61" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="11">
         <f t="shared" si="0"/>
@@ -4982,19 +5695,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L62" s="30" t="s">
+      <c r="L62" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M62" s="14">
         <v>0.1</v>
       </c>
-      <c r="N62" s="37">
+      <c r="N62" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O62" s="9"/>
-    </row>
-    <row r="63" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T62" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U62" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V62" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="11">
         <f>ROW(B63) - ROW($B$2)</f>
@@ -5028,19 +5753,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L63" s="30" t="s">
+      <c r="L63" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M63" s="14">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="N63" s="37">
+      <c r="N63" s="35">
         <f t="shared" si="2"/>
         <v>7.4999999999999997E-2</v>
       </c>
       <c r="O63" s="7"/>
-    </row>
-    <row r="64" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T63" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U63" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V63" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="11">
         <f t="shared" si="0"/>
@@ -5074,19 +5811,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L64" s="30" t="s">
+      <c r="L64" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M64" s="14">
         <v>0.1</v>
       </c>
-      <c r="N64" s="37">
+      <c r="N64" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O64" s="9"/>
-    </row>
-    <row r="65" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T64" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U64" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V64" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="11">
         <f t="shared" si="0"/>
@@ -5120,19 +5869,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L65" s="30" t="s">
+      <c r="L65" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M65" s="14">
         <v>0.1</v>
       </c>
-      <c r="N65" s="37">
+      <c r="N65" s="35">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="O65" s="9"/>
-    </row>
-    <row r="66" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T65" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U65" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V65" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="11">
         <f>ROW(B66) - ROW($B$2)</f>
@@ -5166,19 +5927,31 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L66" s="30" t="s">
+      <c r="L66" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M66" s="14">
         <v>0.1</v>
       </c>
-      <c r="N66" s="37">
+      <c r="N66" s="35">
         <f>M66*K66</f>
         <v>1</v>
       </c>
       <c r="O66" s="9"/>
-    </row>
-    <row r="67" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T66" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U66" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V66" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="11">
         <f t="shared" si="0"/>
@@ -5212,19 +5985,31 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L67" s="30" t="s">
+      <c r="L67" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M67" s="14">
         <v>0.1</v>
       </c>
-      <c r="N67" s="37">
+      <c r="N67" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O67" s="9"/>
-    </row>
-    <row r="68" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T67" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U67" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V67" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="11">
         <f>ROW(B68) - ROW($B$2)</f>
@@ -5258,19 +6043,31 @@
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="L68" s="30" t="s">
+      <c r="L68" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M68" s="14">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="N68" s="37">
+      <c r="N68" s="35">
         <f t="shared" si="2"/>
         <v>0.44999999999999996</v>
       </c>
       <c r="O68" s="7"/>
-    </row>
-    <row r="69" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T68" t="b">
+        <f t="shared" ref="T68:T95" si="8">IF(Q68=D68,TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="U68" t="b">
+        <f t="shared" ref="U68:U95" si="9">IF(R68=G68,TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="V68" t="b">
+        <f t="shared" ref="V68:V95" si="10">IF(S68=J68,TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="11">
         <f t="shared" si="0"/>
@@ -5301,22 +6098,34 @@
         <v>2</v>
       </c>
       <c r="K69" s="7">
-        <f t="shared" ref="K69:K98" si="5">J69*5</f>
+        <f t="shared" ref="K69:K99" si="11">J69*5</f>
         <v>10</v>
       </c>
-      <c r="L69" s="30" t="s">
+      <c r="L69" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M69" s="14">
         <v>1.9E-2</v>
       </c>
-      <c r="N69" s="37">
+      <c r="N69" s="35">
         <f t="shared" si="2"/>
         <v>0.19</v>
       </c>
       <c r="O69" s="9"/>
-    </row>
-    <row r="70" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T69" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U69" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V69" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="11">
         <f>ROW(B70) - ROW($B$2)</f>
@@ -5347,22 +6156,34 @@
         <v>1</v>
       </c>
       <c r="K70" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L70" s="30" t="s">
+      <c r="L70" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M70" s="14">
         <v>0.1</v>
       </c>
-      <c r="N70" s="37">
+      <c r="N70" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O70" s="7"/>
-    </row>
-    <row r="71" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T70" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U70" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V70" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="11">
         <f t="shared" si="0"/>
@@ -5393,22 +6214,34 @@
         <v>1</v>
       </c>
       <c r="K71" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L71" s="30" t="s">
+      <c r="L71" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M71" s="14">
         <v>0.1</v>
       </c>
-      <c r="N71" s="37">
+      <c r="N71" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O71" s="9"/>
-    </row>
-    <row r="72" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T71" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U71" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V71" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="11">
         <f t="shared" si="0"/>
@@ -5439,22 +6272,34 @@
         <v>1</v>
       </c>
       <c r="K72" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L72" s="30" t="s">
+      <c r="L72" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M72" s="14">
         <v>0.14000000000000001</v>
       </c>
-      <c r="N72" s="37">
+      <c r="N72" s="35">
         <f t="shared" si="2"/>
         <v>0.70000000000000007</v>
       </c>
       <c r="O72" s="7"/>
-    </row>
-    <row r="73" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T72" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U72" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V72" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="11">
         <f t="shared" si="0"/>
@@ -5485,22 +6330,34 @@
         <v>1</v>
       </c>
       <c r="K73" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L73" s="30" t="s">
+      <c r="L73" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M73" s="14">
         <v>0.1</v>
       </c>
-      <c r="N73" s="37">
+      <c r="N73" s="35">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="O73" s="7"/>
-    </row>
-    <row r="74" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T73" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U73" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V73" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="11">
         <f>ROW(B74) - ROW($B$2)</f>
@@ -5531,22 +6388,34 @@
         <v>2</v>
       </c>
       <c r="K74" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>10</v>
       </c>
-      <c r="L74" s="30" t="s">
+      <c r="L74" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M74" s="14">
         <v>9.4030000000000002E-2</v>
       </c>
-      <c r="N74" s="37">
+      <c r="N74" s="35">
         <f t="shared" si="2"/>
         <v>0.94030000000000002</v>
       </c>
       <c r="O74" s="7"/>
-    </row>
-    <row r="75" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T74" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U74" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V74" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="11">
         <f t="shared" si="0"/>
@@ -5577,22 +6446,34 @@
         <v>4</v>
       </c>
       <c r="K75" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>20</v>
       </c>
-      <c r="L75" s="30" t="s">
+      <c r="L75" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M75" s="14">
         <v>1.9E-2</v>
       </c>
-      <c r="N75" s="37">
-        <f t="shared" ref="N75:N98" si="6">M75*K75</f>
+      <c r="N75" s="35">
+        <f t="shared" ref="N75:N99" si="12">M75*K75</f>
         <v>0.38</v>
       </c>
       <c r="O75" s="9"/>
-    </row>
-    <row r="76" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T75" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U75" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V75" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
       <c r="B76" s="11">
         <f t="shared" si="0"/>
@@ -5623,22 +6504,34 @@
         <v>2</v>
       </c>
       <c r="K76" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>10</v>
       </c>
-      <c r="L76" s="30" t="s">
+      <c r="L76" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M76" s="14">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="N76" s="37">
-        <f t="shared" si="6"/>
+      <c r="N76" s="35">
+        <f t="shared" si="12"/>
         <v>0.10999999999999999</v>
       </c>
       <c r="O76" s="7"/>
-    </row>
-    <row r="77" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T76" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U76" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V76" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="11">
         <f t="shared" si="0"/>
@@ -5669,22 +6562,34 @@
         <v>4</v>
       </c>
       <c r="K77" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>20</v>
       </c>
-      <c r="L77" s="30" t="s">
+      <c r="L77" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M77" s="14">
         <v>0.16</v>
       </c>
-      <c r="N77" s="37">
-        <f t="shared" si="6"/>
+      <c r="N77" s="35">
+        <f t="shared" si="12"/>
         <v>3.2</v>
       </c>
       <c r="O77" s="7"/>
-    </row>
-    <row r="78" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T77" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U77" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V77" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
       <c r="B78" s="11">
         <f>ROW(B78) - ROW($B$2)</f>
@@ -5715,22 +6620,34 @@
         <v>8</v>
       </c>
       <c r="K78" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>40</v>
       </c>
-      <c r="L78" s="30" t="s">
+      <c r="L78" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M78" s="14">
         <v>0.16</v>
       </c>
-      <c r="N78" s="37">
-        <f t="shared" si="6"/>
+      <c r="N78" s="35">
+        <f t="shared" si="12"/>
         <v>6.4</v>
       </c>
       <c r="O78" s="7"/>
-    </row>
-    <row r="79" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T78" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U78" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V78" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="11">
         <f t="shared" si="0"/>
@@ -5761,22 +6678,34 @@
         <v>8</v>
       </c>
       <c r="K79" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>40</v>
       </c>
-      <c r="L79" s="30" t="s">
+      <c r="L79" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M79" s="14">
         <v>0.16</v>
       </c>
-      <c r="N79" s="37">
-        <f t="shared" si="6"/>
+      <c r="N79" s="35">
+        <f t="shared" si="12"/>
         <v>6.4</v>
       </c>
       <c r="O79" s="7"/>
-    </row>
-    <row r="80" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T79" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U79" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V79" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="11">
         <f>ROW(B80) - ROW($B$2)</f>
@@ -5807,23 +6736,35 @@
         <v>1</v>
       </c>
       <c r="K80" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L80" s="31" t="s">
+      <c r="L80" s="29" t="s">
         <v>336</v>
       </c>
       <c r="M80" s="17" t="s">
         <v>336</v>
       </c>
-      <c r="N80" s="38" t="s">
+      <c r="N80" s="36" t="s">
         <v>336</v>
       </c>
       <c r="O80" s="15" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="81" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T80" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U80" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V80" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="11">
         <f t="shared" si="0"/>
@@ -5854,22 +6795,34 @@
         <v>2</v>
       </c>
       <c r="K81" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>10</v>
       </c>
-      <c r="L81" s="30" t="s">
+      <c r="L81" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M81" s="14">
         <v>0.98299999999999998</v>
       </c>
-      <c r="N81" s="37">
-        <f t="shared" si="6"/>
+      <c r="N81" s="35">
+        <f t="shared" si="12"/>
         <v>9.83</v>
       </c>
       <c r="O81" s="9"/>
-    </row>
-    <row r="82" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T81" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U81" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V81" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
       <c r="B82" s="11">
         <f>ROW(B82) - ROW($B$2)</f>
@@ -5900,22 +6853,34 @@
         <v>1</v>
       </c>
       <c r="K82" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L82" s="30" t="s">
+      <c r="L82" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M82" s="14">
         <v>1.9</v>
       </c>
-      <c r="N82" s="37">
-        <f t="shared" si="6"/>
+      <c r="N82" s="35">
+        <f t="shared" si="12"/>
         <v>9.5</v>
       </c>
       <c r="O82" s="7"/>
-    </row>
-    <row r="83" spans="1:23" s="19" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T82" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U82" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V82" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:26" s="19" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="18"/>
       <c r="B83" s="11">
         <f t="shared" si="0"/>
@@ -5946,17 +6911,17 @@
         <v>1</v>
       </c>
       <c r="K83" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L83" s="30" t="s">
+      <c r="L83" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M83" s="14">
         <v>6.11</v>
       </c>
-      <c r="N83" s="37">
-        <f t="shared" si="6"/>
+      <c r="N83" s="35">
+        <f t="shared" si="12"/>
         <v>30.55</v>
       </c>
       <c r="O83" s="9"/>
@@ -5964,12 +6929,24 @@
       <c r="Q83"/>
       <c r="R83"/>
       <c r="S83"/>
-      <c r="T83"/>
-      <c r="U83"/>
-      <c r="V83"/>
+      <c r="T83" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U83" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V83" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="W83"/>
-    </row>
-    <row r="84" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="X83"/>
+      <c r="Y83"/>
+      <c r="Z83"/>
+    </row>
+    <row r="84" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
       <c r="B84" s="11">
         <f>ROW(B84) - ROW($B$2)</f>
@@ -6000,22 +6977,34 @@
         <v>1</v>
       </c>
       <c r="K84" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L84" s="30" t="s">
+      <c r="L84" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M84" s="14">
         <v>2.41</v>
       </c>
-      <c r="N84" s="37">
-        <f t="shared" si="6"/>
+      <c r="N84" s="35">
+        <f t="shared" si="12"/>
         <v>12.05</v>
       </c>
       <c r="O84" s="7"/>
-    </row>
-    <row r="85" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T84" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U84" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V84" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
       <c r="B85" s="11">
         <f t="shared" si="0"/>
@@ -6046,22 +7035,34 @@
         <v>1</v>
       </c>
       <c r="K85" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L85" s="30" t="s">
+      <c r="L85" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M85" s="14">
         <v>1.43</v>
       </c>
-      <c r="N85" s="37">
-        <f t="shared" si="6"/>
+      <c r="N85" s="35">
+        <f t="shared" si="12"/>
         <v>7.1499999999999995</v>
       </c>
       <c r="O85" s="9"/>
-    </row>
-    <row r="86" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T85" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U85" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V85" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
       <c r="B86" s="11">
         <f>ROW(B86) - ROW($B$2)</f>
@@ -6092,22 +7093,34 @@
         <v>1</v>
       </c>
       <c r="K86" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L86" s="30" t="s">
+      <c r="L86" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M86" s="14">
         <v>2.27</v>
       </c>
-      <c r="N86" s="37">
-        <f t="shared" si="6"/>
+      <c r="N86" s="35">
+        <f t="shared" si="12"/>
         <v>11.35</v>
       </c>
       <c r="O86" s="7"/>
-    </row>
-    <row r="87" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T86" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U86" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V86" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
       <c r="B87" s="11">
         <f t="shared" si="0"/>
@@ -6138,22 +7151,34 @@
         <v>1</v>
       </c>
       <c r="K87" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L87" s="30" t="s">
+      <c r="L87" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M87" s="14">
         <v>1.1599999999999999</v>
       </c>
-      <c r="N87" s="37">
-        <f t="shared" si="6"/>
+      <c r="N87" s="35">
+        <f t="shared" si="12"/>
         <v>5.8</v>
       </c>
       <c r="O87" s="9"/>
-    </row>
-    <row r="88" spans="1:23" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T87" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U87" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V87" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:26" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
       <c r="B88" s="11">
         <f>ROW(B88) - ROW($B$2)</f>
@@ -6184,22 +7209,34 @@
         <v>1</v>
       </c>
       <c r="K88" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L88" s="30" t="s">
+      <c r="L88" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M88" s="14">
         <v>4.66</v>
       </c>
-      <c r="N88" s="37">
-        <f t="shared" si="6"/>
+      <c r="N88" s="35">
+        <f t="shared" si="12"/>
         <v>23.3</v>
       </c>
       <c r="O88" s="7"/>
-    </row>
-    <row r="89" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T88" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U88" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V88" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
       <c r="B89" s="11">
         <f t="shared" si="0"/>
@@ -6230,22 +7267,34 @@
         <v>1</v>
       </c>
       <c r="K89" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L89" s="30" t="s">
+      <c r="L89" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M89" s="14">
         <v>3</v>
       </c>
-      <c r="N89" s="37">
-        <f t="shared" si="6"/>
+      <c r="N89" s="35">
+        <f t="shared" si="12"/>
         <v>15</v>
       </c>
       <c r="O89" s="9"/>
-    </row>
-    <row r="90" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T89" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U89" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V89" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:26" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1"/>
       <c r="B90" s="11">
         <f>ROW(B90) - ROW($B$2)</f>
@@ -6276,22 +7325,34 @@
         <v>1</v>
       </c>
       <c r="K90" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L90" s="30" t="s">
+      <c r="L90" s="28" t="s">
         <v>349</v>
       </c>
       <c r="M90" s="14">
         <v>2.6663999999999999</v>
       </c>
-      <c r="N90" s="37">
-        <f t="shared" si="6"/>
+      <c r="N90" s="35">
+        <f t="shared" si="12"/>
         <v>13.331999999999999</v>
       </c>
       <c r="O90" s="7"/>
-    </row>
-    <row r="91" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T90" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U90" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V90" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1"/>
       <c r="B91" s="11">
         <f t="shared" si="0"/>
@@ -6322,22 +7383,34 @@
         <v>1</v>
       </c>
       <c r="K91" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L91" s="30" t="s">
+      <c r="L91" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M91" s="14">
         <v>4.51</v>
       </c>
-      <c r="N91" s="37">
-        <f t="shared" si="6"/>
+      <c r="N91" s="35">
+        <f t="shared" si="12"/>
         <v>22.549999999999997</v>
       </c>
       <c r="O91" s="9"/>
-    </row>
-    <row r="92" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T91" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U91" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V91" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="1"/>
       <c r="B92" s="11">
         <f>ROW(B92) - ROW($B$2)</f>
@@ -6368,22 +7441,34 @@
         <v>4</v>
       </c>
       <c r="K92" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>20</v>
       </c>
-      <c r="L92" s="30" t="s">
+      <c r="L92" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M92" s="14">
         <v>0.68</v>
       </c>
-      <c r="N92" s="37">
-        <f t="shared" si="6"/>
+      <c r="N92" s="35">
+        <f t="shared" si="12"/>
         <v>13.600000000000001</v>
       </c>
       <c r="O92" s="7"/>
-    </row>
-    <row r="93" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T92" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U92" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V92" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
       <c r="B93" s="11">
         <f t="shared" si="0"/>
@@ -6414,22 +7499,34 @@
         <v>2</v>
       </c>
       <c r="K93" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>10</v>
       </c>
-      <c r="L93" s="30" t="s">
+      <c r="L93" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M93" s="14">
         <v>5.2880000000000003</v>
       </c>
-      <c r="N93" s="37">
-        <f t="shared" si="6"/>
+      <c r="N93" s="35">
+        <f t="shared" si="12"/>
         <v>52.88</v>
       </c>
       <c r="O93" s="9"/>
-    </row>
-    <row r="94" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T93" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U93" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V93" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="1"/>
       <c r="B94" s="11">
         <f>ROW(B94) - ROW($B$2)</f>
@@ -6460,24 +7557,36 @@
         <v>1</v>
       </c>
       <c r="K94" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L94" s="30" t="s">
+      <c r="L94" s="28" t="s">
         <v>337</v>
       </c>
       <c r="M94" s="14">
         <v>0.95</v>
       </c>
-      <c r="N94" s="37">
-        <f t="shared" si="6"/>
+      <c r="N94" s="35">
+        <f t="shared" si="12"/>
         <v>4.75</v>
       </c>
       <c r="O94" s="7"/>
-    </row>
-    <row r="95" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T94" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U94" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V94" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B95" s="11">
-        <f t="shared" ref="B95" si="7">ROW(B95) - ROW($B$2)</f>
+        <f t="shared" ref="B95" si="13">ROW(B95) - ROW($B$2)</f>
         <v>93</v>
       </c>
       <c r="C95" s="13" t="s">
@@ -6503,176 +7612,209 @@
         <v>8</v>
       </c>
       <c r="K95" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>40</v>
       </c>
-      <c r="L95" s="32" t="s">
+      <c r="L95" s="30" t="s">
         <v>337</v>
       </c>
       <c r="M95" s="14">
         <v>2.98</v>
       </c>
-      <c r="N95" s="37">
-        <f t="shared" si="6"/>
+      <c r="N95" s="35">
+        <f t="shared" si="12"/>
         <v>119.2</v>
       </c>
-      <c r="O95" s="23"/>
-    </row>
-    <row r="96" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="O95" s="22"/>
+      <c r="T95" t="b">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U95" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="V95" t="b">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:26" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B96" s="11">
         <f>ROW(B96) - ROW($B$2)</f>
         <v>94</v>
       </c>
-      <c r="C96" s="13" t="s">
+      <c r="C96" s="12" t="s">
         <v>354</v>
       </c>
-      <c r="D96" s="23" t="s">
+      <c r="D96" s="7" t="s">
         <v>336</v>
       </c>
-      <c r="E96" s="23" t="s">
+      <c r="E96" s="7" t="s">
         <v>355</v>
       </c>
-      <c r="F96" s="23" t="s">
+      <c r="F96" s="7" t="s">
         <v>336</v>
       </c>
-      <c r="G96" s="22" t="s">
+      <c r="G96" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="H96" s="23" t="s">
+      <c r="H96" s="7" t="s">
         <v>357</v>
       </c>
-      <c r="I96" s="22" t="s">
+      <c r="I96" s="8" t="s">
         <v>336</v>
       </c>
-      <c r="J96" s="23">
+      <c r="J96" s="7">
         <v>2</v>
       </c>
       <c r="K96" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>10</v>
       </c>
-      <c r="L96" s="32" t="s">
-        <v>337</v>
-      </c>
-      <c r="M96" s="24">
-        <v>0.35</v>
-      </c>
-      <c r="N96" s="39">
-        <f t="shared" si="6"/>
-        <v>3.5</v>
-      </c>
-      <c r="O96" s="23"/>
+      <c r="L96" s="28" t="s">
+        <v>349</v>
+      </c>
+      <c r="M96" s="14">
+        <v>8.3099999999999993E-2</v>
+      </c>
+      <c r="N96" s="35">
+        <f t="shared" si="12"/>
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="O96" s="7"/>
     </row>
     <row r="97" spans="2:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B97" s="11">
-        <f t="shared" ref="B97:B98" si="8">ROW(B97) - ROW($B$2)</f>
+        <f t="shared" ref="B97" si="14">ROW(B97) - ROW($B$2)</f>
         <v>95</v>
       </c>
-      <c r="C97" s="13" t="s">
+      <c r="C97" s="12" t="s">
         <v>354</v>
       </c>
-      <c r="D97" s="9" t="s">
+      <c r="D97" s="7" t="s">
         <v>336</v>
       </c>
-      <c r="E97" s="9" t="s">
+      <c r="E97" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="F97" s="7"/>
+      <c r="G97" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="H97" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="I97" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="J97" s="7">
+        <v>1</v>
+      </c>
+      <c r="K97" s="7">
+        <v>2</v>
+      </c>
+      <c r="L97" s="28" t="s">
+        <v>433</v>
+      </c>
+      <c r="M97" s="14">
+        <v>16.989999999999998</v>
+      </c>
+      <c r="N97" s="35">
+        <f t="shared" si="12"/>
+        <v>33.979999999999997</v>
+      </c>
+      <c r="O97" s="7"/>
+    </row>
+    <row r="98" spans="2:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B98" s="11">
+        <f t="shared" ref="B98:B99" si="15">ROW(B98) - ROW($B$2)</f>
+        <v>96</v>
+      </c>
+      <c r="C98" s="13" t="s">
+        <v>354</v>
+      </c>
+      <c r="D98" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E98" s="9" t="s">
         <v>425</v>
       </c>
-      <c r="F97" s="9" t="s">
+      <c r="F98" s="9" t="s">
         <v>336</v>
       </c>
-      <c r="G97" s="10" t="s">
+      <c r="G98" s="10" t="s">
         <v>424</v>
       </c>
-      <c r="H97" s="9" t="s">
+      <c r="H98" s="9" t="s">
         <v>393</v>
       </c>
-      <c r="I97" s="10" t="s">
+      <c r="I98" s="10" t="s">
         <v>336</v>
       </c>
-      <c r="J97" s="9">
+      <c r="J98" s="9">
         <v>1</v>
       </c>
-      <c r="K97" s="7">
-        <f t="shared" si="5"/>
+      <c r="K98" s="7">
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L97" s="33" t="s">
+      <c r="L98" s="31" t="s">
         <v>349</v>
       </c>
-      <c r="M97" s="35">
+      <c r="M98" s="33">
         <v>0.73499999999999999</v>
       </c>
-      <c r="N97" s="40">
-        <f t="shared" si="6"/>
+      <c r="N98" s="37">
+        <f t="shared" si="12"/>
         <v>3.6749999999999998</v>
       </c>
-      <c r="O97" s="9"/>
-    </row>
-    <row r="98" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B98" s="11">
-        <f t="shared" si="8"/>
-        <v>96</v>
-      </c>
-      <c r="C98" s="25" t="s">
+      <c r="O98" s="9"/>
+    </row>
+    <row r="99" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B99" s="11">
+        <f t="shared" si="15"/>
+        <v>97</v>
+      </c>
+      <c r="C99" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="D98" s="26" t="s">
+      <c r="D99" s="24" t="s">
         <v>336</v>
       </c>
-      <c r="E98" s="26" t="s">
+      <c r="E99" s="24" t="s">
         <v>427</v>
       </c>
-      <c r="F98" s="26" t="s">
+      <c r="F99" s="24" t="s">
         <v>336</v>
       </c>
-      <c r="G98" s="27" t="s">
+      <c r="G99" s="25" t="s">
         <v>426</v>
       </c>
-      <c r="H98" s="26" t="s">
+      <c r="H99" s="24" t="s">
         <v>394</v>
       </c>
-      <c r="I98" s="27" t="s">
+      <c r="I99" s="25" t="s">
         <v>336</v>
       </c>
-      <c r="J98" s="26">
+      <c r="J99" s="24">
         <v>1</v>
       </c>
-      <c r="K98" s="7">
-        <f t="shared" si="5"/>
+      <c r="K99" s="7">
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="L98" s="34" t="s">
+      <c r="L99" s="32" t="s">
         <v>349</v>
       </c>
-      <c r="M98" s="36">
+      <c r="M99" s="34">
         <v>1.2457</v>
       </c>
-      <c r="N98" s="41">
-        <f t="shared" si="6"/>
+      <c r="N99" s="38">
+        <f t="shared" si="12"/>
         <v>6.2285000000000004</v>
       </c>
-      <c r="O98" s="26"/>
-    </row>
-    <row r="99" spans="2:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B99" s="1"/>
-      <c r="C99" s="1"/>
-      <c r="D99" s="1"/>
-      <c r="E99" s="1"/>
-      <c r="F99" s="1"/>
-      <c r="G99" s="1"/>
-      <c r="H99" s="1"/>
-      <c r="I99" s="1"/>
-      <c r="J99" s="1"/>
-      <c r="K99" s="43" t="s">
-        <v>350</v>
-      </c>
-      <c r="L99" s="44"/>
-      <c r="M99" s="45"/>
-      <c r="N99" s="21">
-        <f>SUM(N10:N98)</f>
-        <v>677.73879999999997</v>
-      </c>
-      <c r="O99" s="1"/>
+      <c r="O99" s="24"/>
     </row>
     <row r="100" spans="2:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B100" s="1"/>
@@ -6684,22 +7826,43 @@
       <c r="H100" s="1"/>
       <c r="I100" s="1"/>
       <c r="J100" s="1"/>
-      <c r="K100" s="46" t="s">
+      <c r="K100" s="45" t="s">
+        <v>350</v>
+      </c>
+      <c r="L100" s="46"/>
+      <c r="M100" s="47"/>
+      <c r="N100" s="21">
+        <f>SUM(N10:N99)</f>
+        <v>709.0498</v>
+      </c>
+      <c r="O100" s="1"/>
+    </row>
+    <row r="101" spans="2:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B101" s="1"/>
+      <c r="C101" s="1"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="1"/>
+      <c r="F101" s="1"/>
+      <c r="G101" s="1"/>
+      <c r="H101" s="1"/>
+      <c r="I101" s="1"/>
+      <c r="J101" s="1"/>
+      <c r="K101" s="48" t="s">
         <v>348</v>
       </c>
-      <c r="L100" s="47"/>
-      <c r="M100" s="48"/>
-      <c r="N100" s="20">
-        <f>N99/5</f>
-        <v>135.54775999999998</v>
-      </c>
-      <c r="O100" s="1"/>
+      <c r="L101" s="49"/>
+      <c r="M101" s="50"/>
+      <c r="N101" s="20">
+        <f>N100/5</f>
+        <v>141.80995999999999</v>
+      </c>
+      <c r="O101" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="I1:O1"/>
-    <mergeCell ref="K99:M99"/>
     <mergeCell ref="K100:M100"/>
+    <mergeCell ref="K101:M101"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="L3" r:id="rId1"/>
@@ -6777,28 +7940,29 @@
     <hyperlink ref="L46" r:id="rId73"/>
     <hyperlink ref="L90" r:id="rId74"/>
     <hyperlink ref="L37" r:id="rId75"/>
-    <hyperlink ref="L96" r:id="rId76"/>
-    <hyperlink ref="L32" r:id="rId77"/>
-    <hyperlink ref="L76" r:id="rId78"/>
-    <hyperlink ref="L38" r:id="rId79"/>
-    <hyperlink ref="L39" r:id="rId80"/>
-    <hyperlink ref="L72" r:id="rId81"/>
-    <hyperlink ref="L73" r:id="rId82"/>
-    <hyperlink ref="L34" r:id="rId83"/>
-    <hyperlink ref="L65" r:id="rId84"/>
-    <hyperlink ref="L98" r:id="rId85"/>
-    <hyperlink ref="L19" r:id="rId86"/>
-    <hyperlink ref="L20" r:id="rId87"/>
-    <hyperlink ref="L21" r:id="rId88"/>
-    <hyperlink ref="L77" r:id="rId89"/>
-    <hyperlink ref="L78" r:id="rId90"/>
-    <hyperlink ref="L79" r:id="rId91"/>
-    <hyperlink ref="L95" r:id="rId92"/>
-    <hyperlink ref="L97" r:id="rId93"/>
-    <hyperlink ref="L22" r:id="rId94"/>
-    <hyperlink ref="L35" r:id="rId95"/>
+    <hyperlink ref="L32" r:id="rId76"/>
+    <hyperlink ref="L76" r:id="rId77"/>
+    <hyperlink ref="L38" r:id="rId78"/>
+    <hyperlink ref="L39" r:id="rId79"/>
+    <hyperlink ref="L72" r:id="rId80"/>
+    <hyperlink ref="L73" r:id="rId81"/>
+    <hyperlink ref="L34" r:id="rId82"/>
+    <hyperlink ref="L65" r:id="rId83"/>
+    <hyperlink ref="L99" r:id="rId84"/>
+    <hyperlink ref="L19" r:id="rId85"/>
+    <hyperlink ref="L20" r:id="rId86"/>
+    <hyperlink ref="L21" r:id="rId87"/>
+    <hyperlink ref="L77" r:id="rId88"/>
+    <hyperlink ref="L78" r:id="rId89"/>
+    <hyperlink ref="L79" r:id="rId90"/>
+    <hyperlink ref="L95" r:id="rId91"/>
+    <hyperlink ref="L98" r:id="rId92"/>
+    <hyperlink ref="L22" r:id="rId93"/>
+    <hyperlink ref="L35" r:id="rId94"/>
+    <hyperlink ref="L96" r:id="rId95"/>
+    <hyperlink ref="L97" r:id="rId96"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId96"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId97"/>
 </worksheet>
 </file>
</xml_diff>